<commit_message>
Corrige NaN nos preços, remove duplicatas de postos e melhorias de UX
- Remove 5.919 registros duplicados de postos do banco (dados importados 3x)
- Corrige exibição de NaN nos preços: fmtBRL/fmtBRLp agora tratam valores inválidos
- Corrige cálculo de preço médio em _renderTopPostos (parseFloat + guard)
- Adiciona endpoint DELETE /api/postos para limpar todos os postos
- Adiciona botão "Limpar Dados" na aba Postos Cadastrados
- Corrige layout do popup de posto no mapa (botões empilhados verticalmente)
- Move aba Orçamento para logo após Rotograma no menu lateral
- Gera documentação técnica/funcional v2.0 (GestaoFrotas_Documentacao_v2.docx)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/template_abastecimentos.xlsx
+++ b/template_abastecimentos.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,29 +26,22 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00475569"/>
-      <sz val="9"/>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <name val="Calibri"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <i val="1"/>
-      <color rgb="00166534"/>
-      <sz val="10"/>
+      <color rgb="00888888"/>
+      <sz val="9"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -57,17 +50,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F1F5F9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001E40AF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DCFCE7"/>
+        <fgColor rgb="001E3A8A"/>
       </patternFill>
     </fill>
   </fills>
@@ -81,36 +64,31 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00CCCCCC"/>
       </left>
       <right style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00CCCCCC"/>
       </right>
       <top style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00CCCCCC"/>
       </top>
       <bottom style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00CCCCCC"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -476,182 +454,125 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="5" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚠  INSTRUÇÕES: Preencha a partir da linha 4. Não altere os cabeçalhos. Data: dd/mm/yyyy ou yyyy-mm-dd. Hora: HH:MM. Valores numéricos sem símbolo R$.</t>
+          <t>DATA</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>HORA</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>PLACA</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>MOTORISTA</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>COMBUSTÍVEL</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>QUANTIDADE (L)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>VALOR TOTAL (R$)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>HODÔMETRO (km)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>POSTO</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>OBSERVAÇÃO</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="40" customHeight="1">
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>DATA *</t>
+          <t>2025-01-15</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>HORA</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>PLACA *</t>
+          <t>ABC1D23</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>MOTORISTA</t>
+          <t>João da Silva</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>CPF / MATRÍCULA</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>HODÔMETRO (km)</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>POSTO *</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>CNPJ POSTO</t>
-        </is>
+          <t>Diesel S10</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>450</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>52000</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>CIDADE</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>UF</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>COMBUSTÍVEL *</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>VOLUME (L) *</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>R$/L *</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>VALOR TOTAL (R$)</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>OBSERVAÇÕES</t>
-        </is>
-      </c>
+          <t>Posto Ipiranga</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
     </row>
-    <row r="3" ht="40" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>15/03/2026</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>08:30</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>ABC1234</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>João da Silva</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>123.456.789-00</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="n">
-        <v>152340</v>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>Posto Exemplo Ltda</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>00.000.000/0001-00</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>São Paulo</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>Diesel S-10</t>
-        </is>
-      </c>
-      <c r="L3" s="4" t="n">
-        <v>80.5</v>
-      </c>
-      <c r="M3" s="4" t="n">
-        <v>6.289</v>
-      </c>
-      <c r="N3" s="4" t="n">
-        <v>506.27</v>
-      </c>
-      <c r="O3" s="4" t="inlineStr">
-        <is>
-          <t>← LINHA DE EXEMPLO (apague antes de importar)</t>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>⚠ Preencha a partir da linha 2. A linha 2 é um exemplo e pode ser apagada.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A4:J4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>